<commit_message>
checklist: drop stale V3.2 silkscreen-swap warnings; regenerate bilingual PDF
The V4.4 checklist still carried the four V3.2 as-built silkscreen swap
pairs (C6/C18, R33/C25, C46/C47, L14/C30) from the hardcoded
AS_BUILT_SILK_SWAPS table. Current-board dynamic detection reports zero
swaps, so those notes and the unconditional red legend are gone from both
languages. CHECKLIST.pdf now bundles the Chinese and English tables in
one file (English parsed from CHECKLIST.md with a coverage assertion).
</commit_message>
<xml_diff>
--- a/hardware/expansion-board-v4/CHECKLIST.xlsx
+++ b/hardware/expansion-board-v4/CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V4.4 核对清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="V4.4 核对清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'V4.4 核对清单'!$1:$1</definedName>
@@ -40,7 +40,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,11 +50,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD6D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -127,16 +122,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -699,37 +684,33 @@
       <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="19" customHeight="1">
-      <c r="A7" s="6" t="inlineStr"/>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>C6</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>1uF</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>92.1, 97.9</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `C18`</t>
-        </is>
-      </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="2" t="inlineStr"/>
@@ -964,37 +945,33 @@
       <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="19" customHeight="1">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>10uF</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>C_0805_2012Metric</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>74.4, 80.8</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `C6`</t>
-        </is>
-      </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="19" customHeight="1">
       <c r="A17" s="2" t="inlineStr"/>
@@ -1171,37 +1148,33 @@
       <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="6" t="inlineStr"/>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>C25</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>100nF</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>83.2, 71.6</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>B MCU + Flash</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `R33`，尺寸相同会真贴错</t>
-        </is>
-      </c>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
     <row r="24" ht="19" customHeight="1">
       <c r="A24" s="2" t="inlineStr"/>
@@ -1320,37 +1293,33 @@
       <c r="G27" s="5" t="inlineStr"/>
     </row>
     <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="6" t="inlineStr"/>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>C30</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>100pF</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>C_0402_1005Metric</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>102.8, 67.5</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `L14`，尺寸相同会真贴错</t>
-        </is>
-      </c>
+      <c r="G28" s="5" t="inlineStr"/>
     </row>
     <row r="29" ht="19" customHeight="1">
       <c r="A29" s="2" t="inlineStr"/>
@@ -1788,70 +1757,62 @@
       <c r="G43" s="5" t="inlineStr"/>
     </row>
     <row r="44" ht="19" customHeight="1">
-      <c r="A44" s="6" t="inlineStr"/>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>C46</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>3pF</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>104.9, 78.5</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G44" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `C47`，尺寸相同会真贴错</t>
-        </is>
-      </c>
+      <c r="G44" s="5" t="inlineStr"/>
     </row>
     <row r="45" ht="19" customHeight="1">
-      <c r="A45" s="6" t="inlineStr"/>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>C47</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>200pF</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>104.9, 80.4</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `C46`，尺寸相同会真贴错</t>
-        </is>
-      </c>
+      <c r="G45" s="5" t="inlineStr"/>
     </row>
     <row r="46" ht="19" customHeight="1">
       <c r="A46" s="2" t="inlineStr"/>
@@ -3164,62 +3125,62 @@
       <c r="G91" s="5" t="inlineStr"/>
     </row>
     <row r="92" ht="19" customHeight="1">
-      <c r="A92" s="10" t="inlineStr"/>
-      <c r="B92" s="11" t="inlineStr">
+      <c r="A92" s="6" t="inlineStr"/>
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="C92" s="12" t="inlineStr">
+      <c r="C92" s="8" t="inlineStr">
         <is>
           <t>5.1k DNP(带电源版)</t>
         </is>
       </c>
-      <c r="D92" s="12" t="inlineStr">
+      <c r="D92" s="8" t="inlineStr">
         <is>
           <t>R_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E92" s="10" t="inlineStr">
+      <c r="E92" s="6" t="inlineStr">
         <is>
           <t>145.6, 64.8</t>
         </is>
       </c>
-      <c r="F92" s="12" t="inlineStr">
+      <c r="F92" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G92" s="13" t="inlineStr"/>
+      <c r="G92" s="9" t="inlineStr"/>
     </row>
     <row r="93" ht="19" customHeight="1">
-      <c r="A93" s="10" t="inlineStr"/>
-      <c r="B93" s="11" t="inlineStr">
+      <c r="A93" s="6" t="inlineStr"/>
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="C93" s="12" t="inlineStr">
+      <c r="C93" s="8" t="inlineStr">
         <is>
           <t>5.1k DNP(带电源版)</t>
         </is>
       </c>
-      <c r="D93" s="12" t="inlineStr">
+      <c r="D93" s="8" t="inlineStr">
         <is>
           <t>R_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E93" s="10" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>143.6, 64.8</t>
         </is>
       </c>
-      <c r="F93" s="12" t="inlineStr">
+      <c r="F93" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G93" s="13" t="inlineStr"/>
+      <c r="G93" s="9" t="inlineStr"/>
     </row>
     <row r="94" ht="19" customHeight="1">
       <c r="A94" s="2" t="inlineStr"/>
@@ -3483,62 +3444,62 @@
       <c r="G102" s="5" t="inlineStr"/>
     </row>
     <row r="103" ht="19" customHeight="1">
-      <c r="A103" s="10" t="inlineStr"/>
-      <c r="B103" s="11" t="inlineStr">
+      <c r="A103" s="6" t="inlineStr"/>
+      <c r="B103" s="7" t="inlineStr">
         <is>
           <t>R24</t>
         </is>
       </c>
-      <c r="C103" s="12" t="inlineStr">
+      <c r="C103" s="8" t="inlineStr">
         <is>
           <t>0R DNP(旁路外接)</t>
         </is>
       </c>
-      <c r="D103" s="12" t="inlineStr">
+      <c r="D103" s="8" t="inlineStr">
         <is>
           <t>R_0402_1005Metric</t>
         </is>
       </c>
-      <c r="E103" s="10" t="inlineStr">
+      <c r="E103" s="6" t="inlineStr">
         <is>
           <t>101.1, 63.1</t>
         </is>
       </c>
-      <c r="F103" s="12" t="inlineStr">
+      <c r="F103" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G103" s="13" t="inlineStr"/>
+      <c r="G103" s="9" t="inlineStr"/>
     </row>
     <row r="104" ht="19" customHeight="1">
-      <c r="A104" s="10" t="inlineStr"/>
-      <c r="B104" s="11" t="inlineStr">
+      <c r="A104" s="6" t="inlineStr"/>
+      <c r="B104" s="7" t="inlineStr">
         <is>
           <t>R25</t>
         </is>
       </c>
-      <c r="C104" s="12" t="inlineStr">
+      <c r="C104" s="8" t="inlineStr">
         <is>
           <t>0R DNP(旁路板载)</t>
         </is>
       </c>
-      <c r="D104" s="12" t="inlineStr">
+      <c r="D104" s="8" t="inlineStr">
         <is>
           <t>R_0402_1005Metric</t>
         </is>
       </c>
-      <c r="E104" s="10" t="inlineStr">
+      <c r="E104" s="6" t="inlineStr">
         <is>
           <t>95.5, 62.9</t>
         </is>
       </c>
-      <c r="F104" s="12" t="inlineStr">
+      <c r="F104" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G104" s="13" t="inlineStr"/>
+      <c r="G104" s="9" t="inlineStr"/>
     </row>
     <row r="105" ht="19" customHeight="1">
       <c r="A105" s="2" t="inlineStr"/>
@@ -3599,33 +3560,33 @@
       <c r="G106" s="5" t="inlineStr"/>
     </row>
     <row r="107" ht="19" customHeight="1">
-      <c r="A107" s="10" t="inlineStr"/>
-      <c r="B107" s="11" t="inlineStr">
+      <c r="A107" s="6" t="inlineStr"/>
+      <c r="B107" s="7" t="inlineStr">
         <is>
           <t>R30</t>
         </is>
       </c>
-      <c r="C107" s="12" t="inlineStr">
+      <c r="C107" s="8" t="inlineStr">
         <is>
           <t>1k DNP</t>
         </is>
       </c>
-      <c r="D107" s="12" t="inlineStr">
+      <c r="D107" s="8" t="inlineStr">
         <is>
           <t>R_0402_1005Metric</t>
         </is>
       </c>
-      <c r="E107" s="10" t="inlineStr">
+      <c r="E107" s="6" t="inlineStr">
         <is>
           <t>96.8, 77.2</t>
         </is>
       </c>
-      <c r="F107" s="12" t="inlineStr">
+      <c r="F107" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G107" s="13" t="inlineStr"/>
+      <c r="G107" s="9" t="inlineStr"/>
     </row>
     <row r="108" ht="19" customHeight="1">
       <c r="A108" s="2" t="inlineStr"/>
@@ -3686,37 +3647,33 @@
       <c r="G109" s="5" t="inlineStr"/>
     </row>
     <row r="110" ht="19" customHeight="1">
-      <c r="A110" s="6" t="inlineStr"/>
-      <c r="B110" s="7" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr"/>
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>R33</t>
         </is>
       </c>
-      <c r="C110" s="8" t="inlineStr">
+      <c r="C110" s="4" t="inlineStr">
         <is>
           <t>100k</t>
         </is>
       </c>
-      <c r="D110" s="8" t="inlineStr">
+      <c r="D110" s="4" t="inlineStr">
         <is>
           <t>R_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr">
+      <c r="E110" s="2" t="inlineStr">
         <is>
           <t>100.9, 82.7</t>
         </is>
       </c>
-      <c r="F110" s="8" t="inlineStr">
+      <c r="F110" s="4" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G110" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `C25`，尺寸相同会真贴错</t>
-        </is>
-      </c>
+      <c r="G110" s="5" t="inlineStr"/>
     </row>
     <row r="111" ht="19" customHeight="1">
       <c r="A111" s="2" t="inlineStr"/>
@@ -3777,33 +3734,33 @@
       <c r="G112" s="5" t="inlineStr"/>
     </row>
     <row r="113" ht="19" customHeight="1">
-      <c r="A113" s="10" t="inlineStr"/>
-      <c r="B113" s="11" t="inlineStr">
+      <c r="A113" s="6" t="inlineStr"/>
+      <c r="B113" s="7" t="inlineStr">
         <is>
           <t>R36</t>
         </is>
       </c>
-      <c r="C113" s="12" t="inlineStr">
+      <c r="C113" s="8" t="inlineStr">
         <is>
           <t>1k DNP</t>
         </is>
       </c>
-      <c r="D113" s="12" t="inlineStr">
+      <c r="D113" s="8" t="inlineStr">
         <is>
           <t>R_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E113" s="10" t="inlineStr">
+      <c r="E113" s="6" t="inlineStr">
         <is>
           <t>96.5, 81.8</t>
         </is>
       </c>
-      <c r="F113" s="12" t="inlineStr">
+      <c r="F113" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G113" s="13" t="inlineStr"/>
+      <c r="G113" s="9" t="inlineStr"/>
     </row>
     <row r="114" ht="19" customHeight="1">
       <c r="A114" s="2" t="inlineStr"/>
@@ -4677,37 +4634,33 @@
       <c r="G144" s="5" t="inlineStr"/>
     </row>
     <row r="145" ht="19" customHeight="1">
-      <c r="A145" s="6" t="inlineStr"/>
-      <c r="B145" s="7" t="inlineStr">
+      <c r="A145" s="2" t="inlineStr"/>
+      <c r="B145" s="3" t="inlineStr">
         <is>
           <t>L14</t>
         </is>
       </c>
-      <c r="C145" s="8" t="inlineStr">
+      <c r="C145" s="4" t="inlineStr">
         <is>
           <t>100nH</t>
         </is>
       </c>
-      <c r="D145" s="8" t="inlineStr">
+      <c r="D145" s="4" t="inlineStr">
         <is>
           <t>L_0402_1005Metric</t>
         </is>
       </c>
-      <c r="E145" s="6" t="inlineStr">
+      <c r="E145" s="2" t="inlineStr">
         <is>
           <t>101.1, 70.6</t>
         </is>
       </c>
-      <c r="F145" s="8" t="inlineStr">
+      <c r="F145" s="4" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G145" s="9" t="inlineStr">
-        <is>
-          <t>板上印着 `C30`，尺寸相同会真贴错</t>
-        </is>
-      </c>
+      <c r="G145" s="5" t="inlineStr"/>
     </row>
     <row r="146" ht="19" customHeight="1">
       <c r="A146" s="2" t="inlineStr"/>
@@ -5149,627 +5102,627 @@
     </row>
     <row r="164" ht="19" customHeight="1"/>
     <row r="165" ht="19" customHeight="1">
-      <c r="A165" s="14" t="inlineStr"/>
-      <c r="B165" s="15" t="inlineStr">
+      <c r="A165" s="10" t="inlineStr"/>
+      <c r="B165" s="11" t="inlineStr">
         <is>
           <t>U1</t>
         </is>
       </c>
-      <c r="C165" s="16" t="inlineStr">
+      <c r="C165" s="12" t="inlineStr">
         <is>
           <t>ME6211C33M5</t>
         </is>
       </c>
-      <c r="D165" s="16" t="inlineStr">
+      <c r="D165" s="12" t="inlineStr">
         <is>
           <t>SOT-23-5</t>
         </is>
       </c>
-      <c r="E165" s="14" t="inlineStr">
+      <c r="E165" s="10" t="inlineStr">
         <is>
           <t>74.7, 97.8</t>
         </is>
       </c>
-      <c r="F165" s="16" t="inlineStr">
+      <c r="F165" s="12" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G165" s="17" t="inlineStr">
+      <c r="G165" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="166" ht="19" customHeight="1">
-      <c r="A166" s="14" t="inlineStr"/>
-      <c r="B166" s="15" t="inlineStr">
+      <c r="A166" s="10" t="inlineStr"/>
+      <c r="B166" s="11" t="inlineStr">
         <is>
           <t>U2</t>
         </is>
       </c>
-      <c r="C166" s="16" t="inlineStr">
+      <c r="C166" s="12" t="inlineStr">
         <is>
           <t>TPS7A2033PDBVR</t>
         </is>
       </c>
-      <c r="D166" s="16" t="inlineStr">
+      <c r="D166" s="12" t="inlineStr">
         <is>
           <t>SOT-23-5</t>
         </is>
       </c>
-      <c r="E166" s="14" t="inlineStr">
+      <c r="E166" s="10" t="inlineStr">
         <is>
           <t>82.3, 97.8</t>
         </is>
       </c>
-      <c r="F166" s="16" t="inlineStr">
+      <c r="F166" s="12" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G166" s="17" t="inlineStr">
+      <c r="G166" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="167" ht="19" customHeight="1">
-      <c r="A167" s="14" t="inlineStr"/>
-      <c r="B167" s="15" t="inlineStr">
+      <c r="A167" s="10" t="inlineStr"/>
+      <c r="B167" s="11" t="inlineStr">
         <is>
           <t>U3</t>
         </is>
       </c>
-      <c r="C167" s="16" t="inlineStr">
+      <c r="C167" s="12" t="inlineStr">
         <is>
           <t>TPS7A2033PDBVR</t>
         </is>
       </c>
-      <c r="D167" s="16" t="inlineStr">
+      <c r="D167" s="12" t="inlineStr">
         <is>
           <t>SOT-23-5</t>
         </is>
       </c>
-      <c r="E167" s="14" t="inlineStr">
+      <c r="E167" s="10" t="inlineStr">
         <is>
           <t>89.2, 97.8</t>
         </is>
       </c>
-      <c r="F167" s="16" t="inlineStr">
+      <c r="F167" s="12" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G167" s="17" t="inlineStr">
+      <c r="G167" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="168" ht="19" customHeight="1">
-      <c r="A168" s="14" t="inlineStr"/>
-      <c r="B168" s="15" t="inlineStr">
+      <c r="A168" s="10" t="inlineStr"/>
+      <c r="B168" s="11" t="inlineStr">
         <is>
           <t>U4</t>
         </is>
       </c>
-      <c r="C168" s="16" t="inlineStr">
+      <c r="C168" s="12" t="inlineStr">
         <is>
           <t>BNO085</t>
         </is>
       </c>
-      <c r="D168" s="16" t="inlineStr">
+      <c r="D168" s="12" t="inlineStr">
         <is>
           <t>BNO085_LGA-28</t>
         </is>
       </c>
-      <c r="E168" s="14" t="inlineStr">
+      <c r="E168" s="10" t="inlineStr">
         <is>
           <t>59.7, 84.5</t>
         </is>
       </c>
-      <c r="F168" s="16" t="inlineStr">
+      <c r="F168" s="12" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G168" s="17" t="inlineStr">
+      <c r="G168" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="169" ht="19" customHeight="1">
-      <c r="A169" s="14" t="inlineStr"/>
-      <c r="B169" s="15" t="inlineStr">
+      <c r="A169" s="10" t="inlineStr"/>
+      <c r="B169" s="11" t="inlineStr">
         <is>
           <t>U5</t>
         </is>
       </c>
-      <c r="C169" s="16" t="inlineStr">
+      <c r="C169" s="12" t="inlineStr">
         <is>
           <t>BMP388</t>
         </is>
       </c>
-      <c r="D169" s="16" t="inlineStr">
+      <c r="D169" s="12" t="inlineStr">
         <is>
           <t>BMP388_LGA-10</t>
         </is>
       </c>
-      <c r="E169" s="14" t="inlineStr">
+      <c r="E169" s="10" t="inlineStr">
         <is>
           <t>61.0, 88.9</t>
         </is>
       </c>
-      <c r="F169" s="16" t="inlineStr">
+      <c r="F169" s="12" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G169" s="17" t="inlineStr">
+      <c r="G169" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="170" ht="19" customHeight="1">
-      <c r="A170" s="14" t="inlineStr"/>
-      <c r="B170" s="15" t="inlineStr">
+      <c r="A170" s="10" t="inlineStr"/>
+      <c r="B170" s="11" t="inlineStr">
         <is>
           <t>U6</t>
         </is>
       </c>
-      <c r="C170" s="16" t="inlineStr">
+      <c r="C170" s="12" t="inlineStr">
         <is>
           <t>QMC5883P</t>
         </is>
       </c>
-      <c r="D170" s="16" t="inlineStr">
+      <c r="D170" s="12" t="inlineStr">
         <is>
           <t>LGA-16_3x3mm_P0.5mm</t>
         </is>
       </c>
-      <c r="E170" s="14" t="inlineStr">
+      <c r="E170" s="10" t="inlineStr">
         <is>
           <t>59.7, 96.5</t>
         </is>
       </c>
-      <c r="F170" s="16" t="inlineStr">
+      <c r="F170" s="12" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G170" s="17" t="inlineStr">
+      <c r="G170" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="171" ht="19" customHeight="1">
-      <c r="A171" s="14" t="inlineStr"/>
-      <c r="B171" s="15" t="inlineStr">
+      <c r="A171" s="10" t="inlineStr"/>
+      <c r="B171" s="11" t="inlineStr">
         <is>
           <t>U7</t>
         </is>
       </c>
-      <c r="C171" s="16" t="inlineStr">
+      <c r="C171" s="12" t="inlineStr">
         <is>
           <t>ATGM336H-6N-74</t>
         </is>
       </c>
-      <c r="D171" s="16" t="inlineStr">
+      <c r="D171" s="12" t="inlineStr">
         <is>
           <t>ATGM336H_LCC-18</t>
         </is>
       </c>
-      <c r="E171" s="14" t="inlineStr">
+      <c r="E171" s="10" t="inlineStr">
         <is>
           <t>73.7, 89.1</t>
         </is>
       </c>
-      <c r="F171" s="16" t="inlineStr">
+      <c r="F171" s="12" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G171" s="17" t="inlineStr">
+      <c r="G171" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="172" ht="19" customHeight="1">
-      <c r="A172" s="14" t="inlineStr"/>
-      <c r="B172" s="15" t="inlineStr">
+      <c r="A172" s="10" t="inlineStr"/>
+      <c r="B172" s="11" t="inlineStr">
         <is>
           <t>U8</t>
         </is>
       </c>
-      <c r="C172" s="16" t="inlineStr">
+      <c r="C172" s="12" t="inlineStr">
         <is>
           <t>RP2040</t>
         </is>
       </c>
-      <c r="D172" s="16" t="inlineStr">
+      <c r="D172" s="12" t="inlineStr">
         <is>
           <t>QFN-56-1EP_7x7mm_P0.4mm_EP3.2x3.2mm</t>
         </is>
       </c>
-      <c r="E172" s="14" t="inlineStr">
+      <c r="E172" s="10" t="inlineStr">
         <is>
           <t>86.4, 76.9</t>
         </is>
       </c>
-      <c r="F172" s="16" t="inlineStr">
+      <c r="F172" s="12" t="inlineStr">
         <is>
           <t>B MCU + Flash</t>
         </is>
       </c>
-      <c r="G172" s="17" t="inlineStr">
+      <c r="G172" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="173" ht="19" customHeight="1">
-      <c r="A173" s="14" t="inlineStr"/>
-      <c r="B173" s="15" t="inlineStr">
+      <c r="A173" s="10" t="inlineStr"/>
+      <c r="B173" s="11" t="inlineStr">
         <is>
           <t>U9</t>
         </is>
       </c>
-      <c r="C173" s="16" t="inlineStr">
+      <c r="C173" s="12" t="inlineStr">
         <is>
           <t>W25Q128JVSIQ</t>
         </is>
       </c>
-      <c r="D173" s="16" t="inlineStr">
+      <c r="D173" s="12" t="inlineStr">
         <is>
           <t>SOIC-8_5.3x5.3mm_P1.27mm</t>
         </is>
       </c>
-      <c r="E173" s="14" t="inlineStr">
+      <c r="E173" s="10" t="inlineStr">
         <is>
           <t>93.7, 85.9</t>
         </is>
       </c>
-      <c r="F173" s="16" t="inlineStr">
+      <c r="F173" s="12" t="inlineStr">
         <is>
           <t>B MCU + Flash</t>
         </is>
       </c>
-      <c r="G173" s="17" t="inlineStr">
+      <c r="G173" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="174" ht="19" customHeight="1">
-      <c r="A174" s="14" t="inlineStr"/>
-      <c r="B174" s="15" t="inlineStr">
+      <c r="A174" s="10" t="inlineStr"/>
+      <c r="B174" s="11" t="inlineStr">
         <is>
           <t>U10</t>
         </is>
       </c>
-      <c r="C174" s="16" t="inlineStr">
+      <c r="C174" s="12" t="inlineStr">
         <is>
           <t>CC1312R1F3RGZR</t>
         </is>
       </c>
-      <c r="D174" s="16" t="inlineStr">
+      <c r="D174" s="12" t="inlineStr">
         <is>
           <t>QFN-48-1EP_7x7mm_P0.5mm_EP5.15x5.15mm</t>
         </is>
       </c>
-      <c r="E174" s="14" t="inlineStr">
+      <c r="E174" s="10" t="inlineStr">
         <is>
           <t>104.5, 92.0</t>
         </is>
       </c>
-      <c r="F174" s="16" t="inlineStr">
+      <c r="F174" s="12" t="inlineStr">
         <is>
           <t>D 978 收发</t>
         </is>
       </c>
-      <c r="G174" s="17" t="inlineStr">
+      <c r="G174" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="175" ht="19" customHeight="1">
-      <c r="A175" s="14" t="inlineStr"/>
-      <c r="B175" s="15" t="inlineStr">
+      <c r="A175" s="10" t="inlineStr"/>
+      <c r="B175" s="11" t="inlineStr">
         <is>
           <t>U11</t>
         </is>
       </c>
-      <c r="C175" s="16" t="inlineStr">
+      <c r="C175" s="12" t="inlineStr">
         <is>
           <t>QPL9547TR7</t>
         </is>
       </c>
-      <c r="D175" s="16" t="inlineStr">
+      <c r="D175" s="12" t="inlineStr">
         <is>
           <t>DFN-8-1EP_2x2mm_P0.5mm_EP0.86x1.55mm</t>
         </is>
       </c>
-      <c r="E175" s="14" t="inlineStr">
+      <c r="E175" s="10" t="inlineStr">
         <is>
           <t>107.7, 61.9</t>
         </is>
       </c>
-      <c r="F175" s="16" t="inlineStr">
+      <c r="F175" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G175" s="17" t="inlineStr">
+      <c r="G175" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="176" ht="19" customHeight="1">
-      <c r="A176" s="14" t="inlineStr"/>
-      <c r="B176" s="15" t="inlineStr">
+      <c r="A176" s="10" t="inlineStr"/>
+      <c r="B176" s="11" t="inlineStr">
         <is>
           <t>U12</t>
         </is>
       </c>
-      <c r="C176" s="16" t="inlineStr">
+      <c r="C176" s="12" t="inlineStr">
         <is>
           <t>BGA2817</t>
         </is>
       </c>
-      <c r="D176" s="16" t="inlineStr">
+      <c r="D176" s="12" t="inlineStr">
         <is>
           <t>SOT-363_SC-70-6</t>
         </is>
       </c>
-      <c r="E176" s="14" t="inlineStr">
+      <c r="E176" s="10" t="inlineStr">
         <is>
           <t>117.1, 62.5</t>
         </is>
       </c>
-      <c r="F176" s="16" t="inlineStr">
+      <c r="F176" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G176" s="17" t="inlineStr">
+      <c r="G176" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="177" ht="19" customHeight="1">
-      <c r="A177" s="14" t="inlineStr"/>
-      <c r="B177" s="15" t="inlineStr">
+      <c r="A177" s="10" t="inlineStr"/>
+      <c r="B177" s="11" t="inlineStr">
         <is>
           <t>U14</t>
         </is>
       </c>
-      <c r="C177" s="16" t="inlineStr">
+      <c r="C177" s="12" t="inlineStr">
         <is>
           <t>AD8313ARMZ</t>
         </is>
       </c>
-      <c r="D177" s="16" t="inlineStr">
+      <c r="D177" s="12" t="inlineStr">
         <is>
           <t>MSOP-8_3x3mm_P0.65mm</t>
         </is>
       </c>
-      <c r="E177" s="14" t="inlineStr">
+      <c r="E177" s="10" t="inlineStr">
         <is>
           <t>111.1, 73.4</t>
         </is>
       </c>
-      <c r="F177" s="16" t="inlineStr">
+      <c r="F177" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G177" s="17" t="inlineStr">
+      <c r="G177" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="178" ht="19" customHeight="1">
-      <c r="A178" s="14" t="inlineStr"/>
-      <c r="B178" s="15" t="inlineStr">
+      <c r="A178" s="10" t="inlineStr"/>
+      <c r="B178" s="11" t="inlineStr">
         <is>
           <t>U15</t>
         </is>
       </c>
-      <c r="C178" s="16" t="inlineStr">
+      <c r="C178" s="12" t="inlineStr">
         <is>
           <t>TLV3501(TOKMAS)</t>
         </is>
       </c>
-      <c r="D178" s="16" t="inlineStr">
+      <c r="D178" s="12" t="inlineStr">
         <is>
           <t>SOT-23-6</t>
         </is>
       </c>
-      <c r="E178" s="14" t="inlineStr">
+      <c r="E178" s="10" t="inlineStr">
         <is>
           <t>100.6, 79.5</t>
         </is>
       </c>
-      <c r="F178" s="16" t="inlineStr">
+      <c r="F178" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G178" s="17" t="inlineStr">
+      <c r="G178" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="179" ht="19" customHeight="1">
-      <c r="A179" s="14" t="inlineStr"/>
-      <c r="B179" s="15" t="inlineStr">
+      <c r="A179" s="10" t="inlineStr"/>
+      <c r="B179" s="11" t="inlineStr">
         <is>
           <t>U16</t>
         </is>
       </c>
-      <c r="C179" s="16" t="inlineStr">
+      <c r="C179" s="12" t="inlineStr">
         <is>
           <t>XA17-G4K</t>
         </is>
       </c>
-      <c r="D179" s="16" t="inlineStr">
+      <c r="D179" s="12" t="inlineStr">
         <is>
           <t>SOT-363_SC-70-6</t>
         </is>
       </c>
-      <c r="E179" s="14" t="inlineStr">
+      <c r="E179" s="10" t="inlineStr">
         <is>
           <t>98.0, 62.9</t>
         </is>
       </c>
-      <c r="F179" s="16" t="inlineStr">
+      <c r="F179" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G179" s="17" t="inlineStr">
+      <c r="G179" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="180" ht="19" customHeight="1">
-      <c r="A180" s="14" t="inlineStr"/>
-      <c r="B180" s="15" t="inlineStr">
+      <c r="A180" s="10" t="inlineStr"/>
+      <c r="B180" s="11" t="inlineStr">
         <is>
           <t>U17</t>
         </is>
       </c>
-      <c r="C180" s="16" t="inlineStr">
+      <c r="C180" s="12" t="inlineStr">
         <is>
           <t>XA17-G4K</t>
         </is>
       </c>
-      <c r="D180" s="16" t="inlineStr">
+      <c r="D180" s="12" t="inlineStr">
         <is>
           <t>SOT-363_SC-70-6</t>
         </is>
       </c>
-      <c r="E180" s="14" t="inlineStr">
+      <c r="E180" s="10" t="inlineStr">
         <is>
           <t>68.6, 78.1</t>
         </is>
       </c>
-      <c r="F180" s="16" t="inlineStr">
+      <c r="F180" s="12" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G180" s="17" t="inlineStr">
+      <c r="G180" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="181" ht="19" customHeight="1">
-      <c r="A181" s="14" t="inlineStr"/>
-      <c r="B181" s="15" t="inlineStr">
+      <c r="A181" s="10" t="inlineStr"/>
+      <c r="B181" s="11" t="inlineStr">
         <is>
           <t>U18</t>
         </is>
       </c>
-      <c r="C181" s="16" t="inlineStr">
+      <c r="C181" s="12" t="inlineStr">
         <is>
           <t>CH224K</t>
         </is>
       </c>
-      <c r="D181" s="16" t="inlineStr">
+      <c r="D181" s="12" t="inlineStr">
         <is>
           <t>CH224K_ESSOP-10</t>
         </is>
       </c>
-      <c r="E181" s="14" t="inlineStr">
+      <c r="E181" s="10" t="inlineStr">
         <is>
           <t>132.5, 68.6</t>
         </is>
       </c>
-      <c r="F181" s="16" t="inlineStr">
+      <c r="F181" s="12" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G181" s="17" t="inlineStr">
+      <c r="G181" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="182" ht="19" customHeight="1">
-      <c r="A182" s="14" t="inlineStr"/>
-      <c r="B182" s="15" t="inlineStr">
+      <c r="A182" s="10" t="inlineStr"/>
+      <c r="B182" s="11" t="inlineStr">
         <is>
           <t>U19</t>
         </is>
       </c>
-      <c r="C182" s="16" t="inlineStr">
+      <c r="C182" s="12" t="inlineStr">
         <is>
           <t>SY6970</t>
         </is>
       </c>
-      <c r="D182" s="16" t="inlineStr">
+      <c r="D182" s="12" t="inlineStr">
         <is>
           <t>QFN-24-1EP_4x4mm_P0.5mm_EP2.6x2.6mm_ThermalVias</t>
         </is>
       </c>
-      <c r="E182" s="14" t="inlineStr">
+      <c r="E182" s="10" t="inlineStr">
         <is>
           <t>134.5, 83.7</t>
         </is>
       </c>
-      <c r="F182" s="16" t="inlineStr">
+      <c r="F182" s="12" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G182" s="17" t="inlineStr">
+      <c r="G182" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
       </c>
     </row>
     <row r="183" ht="19" customHeight="1">
-      <c r="A183" s="14" t="inlineStr"/>
-      <c r="B183" s="15" t="inlineStr">
+      <c r="A183" s="10" t="inlineStr"/>
+      <c r="B183" s="11" t="inlineStr">
         <is>
           <t>U20</t>
         </is>
       </c>
-      <c r="C183" s="16" t="inlineStr">
+      <c r="C183" s="12" t="inlineStr">
         <is>
           <t>SY7069</t>
         </is>
       </c>
-      <c r="D183" s="16" t="inlineStr">
+      <c r="D183" s="12" t="inlineStr">
         <is>
           <t>TSOT-23-6</t>
         </is>
       </c>
-      <c r="E183" s="14" t="inlineStr">
+      <c r="E183" s="10" t="inlineStr">
         <is>
           <t>139.2, 95.0</t>
         </is>
       </c>
-      <c r="F183" s="16" t="inlineStr">
+      <c r="F183" s="12" t="inlineStr">
         <is>
           <t>A 电源</t>
         </is>
       </c>
-      <c r="G183" s="17" t="inlineStr">
+      <c r="G183" s="13" t="inlineStr">
         <is>
           <t>认 pin1（缺角/圆点）</t>
         </is>
@@ -5777,66 +5730,66 @@
     </row>
     <row r="184" ht="19" customHeight="1"/>
     <row r="185" ht="19" customHeight="1">
-      <c r="A185" s="14" t="inlineStr"/>
-      <c r="B185" s="15" t="inlineStr">
+      <c r="A185" s="10" t="inlineStr"/>
+      <c r="B185" s="11" t="inlineStr">
         <is>
           <t>FL1</t>
         </is>
       </c>
-      <c r="C185" s="16" t="inlineStr">
+      <c r="C185" s="12" t="inlineStr">
         <is>
           <t>TA0970A</t>
         </is>
       </c>
-      <c r="D185" s="16" t="inlineStr">
+      <c r="D185" s="12" t="inlineStr">
         <is>
           <t>TA0970A_SMD3838-6</t>
         </is>
       </c>
-      <c r="E185" s="14" t="inlineStr">
+      <c r="E185" s="10" t="inlineStr">
         <is>
           <t>112.0, 65.5</t>
         </is>
       </c>
-      <c r="F185" s="16" t="inlineStr">
+      <c r="F185" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G185" s="17" t="inlineStr">
+      <c r="G185" s="13" t="inlineStr">
         <is>
           <t>SAW 滤波器分输入输出，贴反不工作</t>
         </is>
       </c>
     </row>
     <row r="186" ht="19" customHeight="1">
-      <c r="A186" s="14" t="inlineStr"/>
-      <c r="B186" s="15" t="inlineStr">
+      <c r="A186" s="10" t="inlineStr"/>
+      <c r="B186" s="11" t="inlineStr">
         <is>
           <t>FL2</t>
         </is>
       </c>
-      <c r="C186" s="16" t="inlineStr">
+      <c r="C186" s="12" t="inlineStr">
         <is>
           <t>TA0970A</t>
         </is>
       </c>
-      <c r="D186" s="16" t="inlineStr">
+      <c r="D186" s="12" t="inlineStr">
         <is>
           <t>TA0970A_SMD3838-6</t>
         </is>
       </c>
-      <c r="E186" s="14" t="inlineStr">
+      <c r="E186" s="10" t="inlineStr">
         <is>
           <t>118.4, 66.5</t>
         </is>
       </c>
-      <c r="F186" s="16" t="inlineStr">
+      <c r="F186" s="12" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G186" s="17" t="inlineStr">
+      <c r="G186" s="13" t="inlineStr">
         <is>
           <t>SAW 滤波器分输入输出，贴反不工作</t>
         </is>
@@ -6173,33 +6126,33 @@
     </row>
     <row r="200" ht="19" customHeight="1"/>
     <row r="201" ht="19" customHeight="1">
-      <c r="A201" s="10" t="inlineStr"/>
-      <c r="B201" s="11" t="inlineStr">
+      <c r="A201" s="6" t="inlineStr"/>
+      <c r="B201" s="7" t="inlineStr">
         <is>
           <t>ANT1</t>
         </is>
       </c>
-      <c r="C201" s="12" t="inlineStr">
+      <c r="C201" s="8" t="inlineStr">
         <is>
           <t>IFA_1090</t>
         </is>
       </c>
-      <c r="D201" s="12" t="inlineStr">
+      <c r="D201" s="8" t="inlineStr">
         <is>
           <t>ANT_IFA_1090MHz</t>
         </is>
       </c>
-      <c r="E201" s="10" t="inlineStr">
+      <c r="E201" s="6" t="inlineStr">
         <is>
           <t>79.2, 57.8</t>
         </is>
       </c>
-      <c r="F201" s="12" t="inlineStr">
+      <c r="F201" s="8" t="inlineStr">
         <is>
           <t>不贴（板载天线）</t>
         </is>
       </c>
-      <c r="G201" s="13" t="inlineStr">
+      <c r="G201" s="9" t="inlineStr">
         <is>
           <t>50.0mm外包络/48.5mm中心线；V4.0装盒实测1082.5MHz、SWR 1.09</t>
         </is>
@@ -6207,66 +6160,66 @@
     </row>
     <row r="202" ht="19" customHeight="1"/>
     <row r="203" ht="19" customHeight="1">
-      <c r="A203" s="10" t="inlineStr"/>
-      <c r="B203" s="11" t="inlineStr">
+      <c r="A203" s="6" t="inlineStr"/>
+      <c r="B203" s="7" t="inlineStr">
         <is>
           <t>ZP1</t>
         </is>
       </c>
-      <c r="C203" s="12" t="inlineStr">
+      <c r="C203" s="8" t="inlineStr">
         <is>
           <t>DNP 并-天线侧</t>
         </is>
       </c>
-      <c r="D203" s="12" t="inlineStr">
+      <c r="D203" s="8" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E203" s="10" t="inlineStr">
+      <c r="E203" s="6" t="inlineStr">
         <is>
           <t>79.2, 63.6</t>
         </is>
       </c>
-      <c r="F203" s="12" t="inlineStr">
+      <c r="F203" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G203" s="13" t="inlineStr">
+      <c r="G203" s="9" t="inlineStr">
         <is>
           <t>默认DNP；V4.0实测直通状态</t>
         </is>
       </c>
     </row>
     <row r="204" ht="19" customHeight="1">
-      <c r="A204" s="10" t="inlineStr"/>
-      <c r="B204" s="11" t="inlineStr">
+      <c r="A204" s="6" t="inlineStr"/>
+      <c r="B204" s="7" t="inlineStr">
         <is>
           <t>ZP2</t>
         </is>
       </c>
-      <c r="C204" s="12" t="inlineStr">
+      <c r="C204" s="8" t="inlineStr">
         <is>
           <t>DNP 并-电台侧</t>
         </is>
       </c>
-      <c r="D204" s="12" t="inlineStr">
+      <c r="D204" s="8" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E204" s="10" t="inlineStr">
+      <c r="E204" s="6" t="inlineStr">
         <is>
           <t>84.2, 63.6</t>
         </is>
       </c>
-      <c r="F204" s="12" t="inlineStr">
+      <c r="F204" s="8" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G204" s="13" t="inlineStr">
+      <c r="G204" s="9" t="inlineStr">
         <is>
           <t>默认DNP；历史HFSS 3.3pF仅作异常复调备选</t>
         </is>
@@ -6308,383 +6261,383 @@
     </row>
     <row r="207" ht="19" customHeight="1"/>
     <row r="208" ht="19" customHeight="1">
-      <c r="A208" s="10" t="inlineStr"/>
-      <c r="B208" s="11" t="inlineStr">
+      <c r="A208" s="6" t="inlineStr"/>
+      <c r="B208" s="7" t="inlineStr">
         <is>
           <t>SW1</t>
         </is>
       </c>
-      <c r="C208" s="12" t="inlineStr">
+      <c r="C208" s="8" t="inlineStr">
         <is>
           <t>RESET短接焊盘</t>
         </is>
       </c>
-      <c r="D208" s="12" t="inlineStr">
+      <c r="D208" s="8" t="inlineStr">
         <is>
           <t>SolderJumper-2_P1.3mm_Open_Pad1.0x1.5mm</t>
         </is>
       </c>
-      <c r="E208" s="10" t="inlineStr">
+      <c r="E208" s="6" t="inlineStr">
         <is>
           <t>51.9, 77.5</t>
         </is>
       </c>
-      <c r="F208" s="12" t="inlineStr">
+      <c r="F208" s="8" t="inlineStr">
         <is>
           <t>不贴（短接焊盘）</t>
         </is>
       </c>
-      <c r="G208" s="13" t="inlineStr"/>
+      <c r="G208" s="9" t="inlineStr"/>
     </row>
     <row r="209" ht="19" customHeight="1">
-      <c r="A209" s="10" t="inlineStr"/>
-      <c r="B209" s="11" t="inlineStr">
+      <c r="A209" s="6" t="inlineStr"/>
+      <c r="B209" s="7" t="inlineStr">
         <is>
           <t>SW2</t>
         </is>
       </c>
-      <c r="C209" s="12" t="inlineStr">
+      <c r="C209" s="8" t="inlineStr">
         <is>
           <t>BOOTSEL短接焊盘</t>
         </is>
       </c>
-      <c r="D209" s="12" t="inlineStr">
+      <c r="D209" s="8" t="inlineStr">
         <is>
           <t>SolderJumper-2_P1.3mm_Open_Pad1.0x1.5mm</t>
         </is>
       </c>
-      <c r="E209" s="10" t="inlineStr">
+      <c r="E209" s="6" t="inlineStr">
         <is>
           <t>51.9, 81.0</t>
         </is>
       </c>
-      <c r="F209" s="12" t="inlineStr">
+      <c r="F209" s="8" t="inlineStr">
         <is>
           <t>不贴（短接焊盘）</t>
         </is>
       </c>
-      <c r="G209" s="13" t="inlineStr"/>
+      <c r="G209" s="9" t="inlineStr"/>
     </row>
     <row r="210" ht="19" customHeight="1"/>
     <row r="211" ht="19" customHeight="1">
-      <c r="A211" s="10" t="inlineStr"/>
-      <c r="B211" s="11" t="inlineStr">
+      <c r="A211" s="6" t="inlineStr"/>
+      <c r="B211" s="7" t="inlineStr">
         <is>
           <t>TP1</t>
         </is>
       </c>
-      <c r="C211" s="12" t="inlineStr">
+      <c r="C211" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D211" s="12" t="inlineStr">
+      <c r="D211" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E211" s="10" t="inlineStr">
+      <c r="E211" s="6" t="inlineStr">
         <is>
           <t>51.9, 86.0</t>
         </is>
       </c>
-      <c r="F211" s="12" t="inlineStr">
+      <c r="F211" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G211" s="13" t="inlineStr"/>
+      <c r="G211" s="9" t="inlineStr"/>
     </row>
     <row r="212" ht="19" customHeight="1">
-      <c r="A212" s="10" t="inlineStr"/>
-      <c r="B212" s="11" t="inlineStr">
+      <c r="A212" s="6" t="inlineStr"/>
+      <c r="B212" s="7" t="inlineStr">
         <is>
           <t>TP2</t>
         </is>
       </c>
-      <c r="C212" s="12" t="inlineStr">
+      <c r="C212" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D212" s="12" t="inlineStr">
+      <c r="D212" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E212" s="10" t="inlineStr">
+      <c r="E212" s="6" t="inlineStr">
         <is>
           <t>51.9, 88.1</t>
         </is>
       </c>
-      <c r="F212" s="12" t="inlineStr">
+      <c r="F212" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G212" s="13" t="inlineStr"/>
+      <c r="G212" s="9" t="inlineStr"/>
     </row>
     <row r="213" ht="19" customHeight="1">
-      <c r="A213" s="10" t="inlineStr"/>
-      <c r="B213" s="11" t="inlineStr">
+      <c r="A213" s="6" t="inlineStr"/>
+      <c r="B213" s="7" t="inlineStr">
         <is>
           <t>TP3</t>
         </is>
       </c>
-      <c r="C213" s="12" t="inlineStr">
+      <c r="C213" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D213" s="12" t="inlineStr">
+      <c r="D213" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E213" s="10" t="inlineStr">
+      <c r="E213" s="6" t="inlineStr">
         <is>
           <t>51.9, 90.1</t>
         </is>
       </c>
-      <c r="F213" s="12" t="inlineStr">
+      <c r="F213" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G213" s="13" t="inlineStr"/>
+      <c r="G213" s="9" t="inlineStr"/>
     </row>
     <row r="214" ht="19" customHeight="1">
-      <c r="A214" s="10" t="inlineStr"/>
-      <c r="B214" s="11" t="inlineStr">
+      <c r="A214" s="6" t="inlineStr"/>
+      <c r="B214" s="7" t="inlineStr">
         <is>
           <t>TP4</t>
         </is>
       </c>
-      <c r="C214" s="12" t="inlineStr">
+      <c r="C214" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D214" s="12" t="inlineStr">
+      <c r="D214" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E214" s="10" t="inlineStr">
+      <c r="E214" s="6" t="inlineStr">
         <is>
           <t>51.9, 92.1</t>
         </is>
       </c>
-      <c r="F214" s="12" t="inlineStr">
+      <c r="F214" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G214" s="13" t="inlineStr"/>
+      <c r="G214" s="9" t="inlineStr"/>
     </row>
     <row r="215" ht="19" customHeight="1">
-      <c r="A215" s="10" t="inlineStr"/>
-      <c r="B215" s="11" t="inlineStr">
+      <c r="A215" s="6" t="inlineStr"/>
+      <c r="B215" s="7" t="inlineStr">
         <is>
           <t>TP5</t>
         </is>
       </c>
-      <c r="C215" s="12" t="inlineStr">
+      <c r="C215" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D215" s="12" t="inlineStr">
+      <c r="D215" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E215" s="10" t="inlineStr">
+      <c r="E215" s="6" t="inlineStr">
         <is>
           <t>51.9, 94.2</t>
         </is>
       </c>
-      <c r="F215" s="12" t="inlineStr">
+      <c r="F215" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G215" s="13" t="inlineStr"/>
+      <c r="G215" s="9" t="inlineStr"/>
     </row>
     <row r="216" ht="19" customHeight="1">
-      <c r="A216" s="10" t="inlineStr"/>
-      <c r="B216" s="11" t="inlineStr">
+      <c r="A216" s="6" t="inlineStr"/>
+      <c r="B216" s="7" t="inlineStr">
         <is>
           <t>TP6</t>
         </is>
       </c>
-      <c r="C216" s="12" t="inlineStr">
+      <c r="C216" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D216" s="12" t="inlineStr">
+      <c r="D216" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E216" s="10" t="inlineStr">
+      <c r="E216" s="6" t="inlineStr">
         <is>
           <t>51.9, 96.2</t>
         </is>
       </c>
-      <c r="F216" s="12" t="inlineStr">
+      <c r="F216" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G216" s="13" t="inlineStr"/>
+      <c r="G216" s="9" t="inlineStr"/>
     </row>
     <row r="217" ht="19" customHeight="1">
-      <c r="A217" s="10" t="inlineStr"/>
-      <c r="B217" s="11" t="inlineStr">
+      <c r="A217" s="6" t="inlineStr"/>
+      <c r="B217" s="7" t="inlineStr">
         <is>
           <t>TP7</t>
         </is>
       </c>
-      <c r="C217" s="12" t="inlineStr">
+      <c r="C217" s="8" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D217" s="12" t="inlineStr">
+      <c r="D217" s="8" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E217" s="10" t="inlineStr">
+      <c r="E217" s="6" t="inlineStr">
         <is>
           <t>51.9, 98.2</t>
         </is>
       </c>
-      <c r="F217" s="12" t="inlineStr">
+      <c r="F217" s="8" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G217" s="13" t="inlineStr"/>
+      <c r="G217" s="9" t="inlineStr"/>
     </row>
     <row r="218" ht="19" customHeight="1"/>
     <row r="219" ht="19" customHeight="1">
-      <c r="A219" s="10" t="inlineStr"/>
-      <c r="B219" s="11" t="inlineStr">
+      <c r="A219" s="6" t="inlineStr"/>
+      <c r="B219" s="7" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="C219" s="12" t="inlineStr">
+      <c r="C219" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D219" s="12" t="inlineStr">
+      <c r="D219" s="8" t="inlineStr">
         <is>
           <t>MountingHole_2.7mm_M2.5</t>
         </is>
       </c>
-      <c r="E219" s="10" t="inlineStr">
+      <c r="E219" s="6" t="inlineStr">
         <is>
           <t>54.0, 56.0</t>
         </is>
       </c>
-      <c r="F219" s="12" t="inlineStr">
+      <c r="F219" s="8" t="inlineStr">
         <is>
           <t>不贴（安装孔）</t>
         </is>
       </c>
-      <c r="G219" s="13" t="inlineStr"/>
+      <c r="G219" s="9" t="inlineStr"/>
     </row>
     <row r="220" ht="19" customHeight="1">
-      <c r="A220" s="10" t="inlineStr"/>
-      <c r="B220" s="11" t="inlineStr">
+      <c r="A220" s="6" t="inlineStr"/>
+      <c r="B220" s="7" t="inlineStr">
         <is>
           <t>H2</t>
         </is>
       </c>
-      <c r="C220" s="12" t="inlineStr">
+      <c r="C220" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D220" s="12" t="inlineStr">
+      <c r="D220" s="8" t="inlineStr">
         <is>
           <t>MountingHole_2.7mm_M2.5</t>
         </is>
       </c>
-      <c r="E220" s="10" t="inlineStr">
+      <c r="E220" s="6" t="inlineStr">
         <is>
           <t>146.0, 56.0</t>
         </is>
       </c>
-      <c r="F220" s="12" t="inlineStr">
+      <c r="F220" s="8" t="inlineStr">
         <is>
           <t>不贴（安装孔）</t>
         </is>
       </c>
-      <c r="G220" s="13" t="inlineStr"/>
+      <c r="G220" s="9" t="inlineStr"/>
     </row>
     <row r="221" ht="19" customHeight="1">
-      <c r="A221" s="10" t="inlineStr"/>
-      <c r="B221" s="11" t="inlineStr">
+      <c r="A221" s="6" t="inlineStr"/>
+      <c r="B221" s="7" t="inlineStr">
         <is>
           <t>H3</t>
         </is>
       </c>
-      <c r="C221" s="12" t="inlineStr">
+      <c r="C221" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D221" s="12" t="inlineStr">
+      <c r="D221" s="8" t="inlineStr">
         <is>
           <t>MountingHole_2.7mm_M2.5</t>
         </is>
       </c>
-      <c r="E221" s="10" t="inlineStr">
+      <c r="E221" s="6" t="inlineStr">
         <is>
           <t>54.0, 106.0</t>
         </is>
       </c>
-      <c r="F221" s="12" t="inlineStr">
+      <c r="F221" s="8" t="inlineStr">
         <is>
           <t>不贴（安装孔）</t>
         </is>
       </c>
-      <c r="G221" s="13" t="inlineStr"/>
+      <c r="G221" s="9" t="inlineStr"/>
     </row>
     <row r="222" ht="19" customHeight="1">
-      <c r="A222" s="10" t="inlineStr"/>
-      <c r="B222" s="11" t="inlineStr">
+      <c r="A222" s="6" t="inlineStr"/>
+      <c r="B222" s="7" t="inlineStr">
         <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="C222" s="12" t="inlineStr">
+      <c r="C222" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D222" s="12" t="inlineStr">
+      <c r="D222" s="8" t="inlineStr">
         <is>
           <t>MountingHole_2.7mm_M2.5</t>
         </is>
       </c>
-      <c r="E222" s="10" t="inlineStr">
+      <c r="E222" s="6" t="inlineStr">
         <is>
           <t>146.0, 106.0</t>
         </is>
       </c>
-      <c r="F222" s="12" t="inlineStr">
+      <c r="F222" s="8" t="inlineStr">
         <is>
           <t>不贴（安装孔）</t>
         </is>
       </c>
-      <c r="G222" s="13" t="inlineStr"/>
+      <c r="G222" s="9" t="inlineStr"/>
     </row>
     <row r="223" ht="19" customHeight="1"/>
     <row r="224" ht="19" customHeight="1">

</xml_diff>